<commit_message>
Record answers and add installed-size column
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z5pCoVvnUESSHvBHrad3z
</commit_message>
<xml_diff>
--- a/tracker/2250823/Filter_Log.xlsx
+++ b/tracker/2250823/Filter_Log.xlsx
@@ -42,12 +42,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -71,10 +71,10 @@
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -450,7 +450,8 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,7 +484,11 @@
           <t>Phase</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>None (single phase for now)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -510,37 +515,42 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Filter size (W x L x D)</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" s="2" t="inlineStr">
         <is>
           <t>Qty per change</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Filter set installed</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>MERV</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Installed size if different from spec</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -571,6 +581,7 @@
       <c r="F8" t="n">
         <v>8</v>
       </c>
+      <c r="G8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -597,6 +608,7 @@
       <c r="F9" t="n">
         <v>8</v>
       </c>
+      <c r="G9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -623,6 +635,7 @@
       <c r="F10" t="n">
         <v>8</v>
       </c>
+      <c r="G10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -649,6 +662,7 @@
       <c r="F11" t="n">
         <v>8</v>
       </c>
+      <c r="G11" s="3" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -675,6 +689,7 @@
       <c r="F12" t="n">
         <v>8</v>
       </c>
+      <c r="G12" s="3" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -701,6 +716,7 @@
       <c r="F13" t="n">
         <v>8</v>
       </c>
+      <c r="G13" s="3" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -727,6 +743,7 @@
       <c r="F14" t="n">
         <v>8</v>
       </c>
+      <c r="G14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -753,6 +770,7 @@
       <c r="F15" t="n">
         <v>8</v>
       </c>
+      <c r="G15" s="3" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -877,8 +895,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
+      <c r="E20" s="3" t="n"/>
+      <c r="F20" s="3" t="n"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -899,8 +917,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
+      <c r="E21" s="3" t="n"/>
+      <c r="F21" s="3" t="n"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -921,8 +939,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -943,8 +961,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E23" s="2" t="n"/>
-      <c r="F23" s="2" t="n"/>
+      <c r="E23" s="3" t="n"/>
+      <c r="F23" s="3" t="n"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -965,8 +983,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
+      <c r="E24" s="3" t="n"/>
+      <c r="F24" s="3" t="n"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -987,8 +1005,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E25" s="2" t="n"/>
-      <c r="F25" s="2" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1009,8 +1027,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1031,8 +1049,8 @@
           <t>Not replaced</t>
         </is>
       </c>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
+      <c r="E27" s="3" t="n"/>
+      <c r="F27" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
RTU-2B-1 is the unit not started, not 2B-2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014z5pCoVvnUESSHvBHrad3z
</commit_message>
<xml_diff>
--- a/tracker/2250823/Filter_Log.xlsx
+++ b/tracker/2250823/Filter_Log.xlsx
@@ -838,17 +838,13 @@
       <c r="C18" t="n">
         <v>8</v>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Replaced</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>2</v>
-      </c>
-      <c r="F18" t="n">
-        <v>8</v>
-      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Not replaced</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n"/>
+      <c r="F18" s="3" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -864,17 +860,13 @@
       <c r="C19" t="n">
         <v>4</v>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Replaced</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>2</v>
-      </c>
-      <c r="F19" t="n">
-        <v>8</v>
-      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>Not replaced</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="n"/>
+      <c r="F19" s="3" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -890,13 +882,17 @@
       <c r="C20" t="n">
         <v>8</v>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Not replaced</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="n"/>
-      <c r="F20" s="3" t="n"/>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Replaced</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -912,13 +908,17 @@
       <c r="C21" t="n">
         <v>4</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Not replaced</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="n"/>
-      <c r="F21" s="3" t="n"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Replaced</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">

</xml_diff>